<commit_message>
Release v1.3.0: correct optical calculations, diagnostics, plots and scientific documentation
Content tree matches tested local release 298057facd7ffddd80b28723b576b6f6789db768.
</commit_message>
<xml_diff>
--- a/examples/01_TiO2_on_BK7_65deg.xlsx
+++ b/examples/01_TiO2_on_BK7_65deg.xlsx
@@ -10,7 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спектр" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Условия" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Спектр'!$A$1:$E$202</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Спектр'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -67,7 +70,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -434,7 +439,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3891,7 +3896,9 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3899,7 +3906,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3908,7 +3915,7 @@
     <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Образец</t>
@@ -3920,7 +3927,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Материал плёнки (априори)</t>
@@ -3932,7 +3939,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Модель дисперсии</t>
@@ -3944,7 +3951,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Справочные параметры</t>
@@ -3952,11 +3959,11 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>A = 255.83, E0 = 4.00 эВ, C = 1.77 эВ, Eg = 3.40 эВ, A_uv = 137.65 эВ², E_uv = 11.0 эВ</t>
+          <t>A = 255.83 эВ, E₀ = 4.00 эВ, C = 1.77 эВ, E_g = 3.40 эВ, A_uv = 137.65 эВ², E_uv = 11.0 эВ</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Подложка</t>
@@ -3968,7 +3975,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="24" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Задняя сторона подложки</t>
@@ -3980,7 +3987,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Угол падения, град</t>
@@ -3990,7 +3997,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="24" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Толщина (номинал), нм</t>
@@ -4000,7 +4007,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="24" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Неопределённость толщины, %</t>
@@ -4012,7 +4019,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Диапазон длин волн, нм</t>
@@ -4024,7 +4031,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Спектральная полоса прибора, нм (FWHM)</t>
@@ -4034,7 +4041,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="24" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Шумовая модель</t>
@@ -4046,19 +4053,19 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Прибор</t>
+          <t>Модель измерения</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>RCE-эллипсометр с ПЗС, все длины волн одновременно; Δ в диапазоне 0–360°; конвенция N = n − ik (Аззам–Башара)</t>
+          <t>Синтетический спектр с независимым гауссовым шумом; σ зависит от длины волны. Δ в диапазоне [0°, 360°); конвенция N = n − ik (Аззам–Башара).</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="56" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Возможные дефекты</t>
@@ -4070,7 +4077,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="56" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Назначение</t>
@@ -4078,11 +4085,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>тестовый файл для приложения: опорный фит однородной плёнки → ИИ по остатку → окончательный фит; истинные параметры — в answer_key.xlsx</t>
+          <t>Учебный спектр, синтезированный tools/gen_examples.js; не измерение физического образца. Опорный фит → классификатор по остатку → окончательный фит; заданные параметры — в answer_key.xlsx.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>